<commit_message>
refactor(product): remove HsnCode property and related database column
- Deleted HsnCode from Product entity and related DTOs
- Removed HsnCode index and column from database via migration
- Updated entity configurations and database model snapshot accordingly
- Adjusted ProductsController and Excel upload parsing to omit HsnCode handling
- Cleaned usages of HsnCode in search and CRUD operations to avoid references
- Ensured backward compatibility with existing data by dropping HsnCode safely
</commit_message>
<xml_diff>
--- a/Frontend/public/Product_Template.xlsx
+++ b/Frontend/public/Product_Template.xlsx
@@ -1,53 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Product Template" sheetId="1" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -66,13 +43,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -397,261 +441,331 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col width="35.83203125" customWidth="1" min="1" max="1"/>
+    <col width="20.83203125" customWidth="1" min="2" max="2"/>
+    <col width="15.83203125" customWidth="1" min="3" max="3"/>
+    <col width="25.83203125" customWidth="1" min="4" max="4"/>
+    <col width="20.83203125" customWidth="1" min="5" max="5"/>
+    <col width="18.83203125" customWidth="1" min="6" max="6"/>
+    <col width="15.83203125" customWidth="1" min="7" max="7"/>
+    <col width="12.83203125" customWidth="1" min="8" max="8"/>
+    <col width="12.83203125" customWidth="1" min="9" max="9"/>
+    <col width="12.83203125" customWidth="1" min="10" max="10"/>
+    <col width="20.83203125" customWidth="1" min="11" max="11"/>
+    <col width="10.83203125" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Product Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>SKU</v>
-      </c>
-      <c r="C1" t="str">
-        <v>HSN Code</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Manufacturer Name</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Commodity Name</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Country of Origin</v>
-      </c>
-      <c r="G1" t="str">
-        <v>MRP Quantity</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Unit Type</v>
-      </c>
-      <c r="I1" t="str">
-        <v>MRP</v>
-      </c>
-      <c r="J1" t="str">
-        <v>USSP</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Best Before (Months)</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Factor</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Product Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Manufacturer Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Commodity Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Country of Origin</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>MRP Quantity</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Unit Type</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MRP</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>USSP</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Best Before (Months)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v>India</v>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v>UNIT</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v>12</v>
-      </c>
-      <c r="L2" t="str">
-        <v>1</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col width="25.83203125" customWidth="1" min="1" max="1"/>
+    <col width="45.83203125" customWidth="1" min="2" max="2"/>
+    <col width="30.83203125" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Example</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Product Name</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Full product name (Required)</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Mechanical Keyboard Pro V2</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Product Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Full product name (Required)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mechanical Keyboard Pro V2</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>SKU</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Unique Stock Keeping Unit code</v>
-      </c>
-      <c r="C3" t="str">
-        <v>KB-001-2024</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Unique Stock Keeping Unit code</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KB-001-2024</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>HSN Code</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Harmonized System of Nomenclature code</v>
-      </c>
-      <c r="C4" t="str">
-        <v>84716060</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Manufacturer Name</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Manufacturer name (must exist in system)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KeyChron</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>Manufacturer Name</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Manufacturer name (must exist in system)</v>
-      </c>
-      <c r="C5" t="str">
-        <v>KeyChron</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Commodity Name</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Category/Commodity name (must exist in system)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>Commodity Name</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Category/Commodity name (must exist in system)</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Electronics</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Country of Origin</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Country where product is manufactured</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>India, China, USA</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>Country of Origin</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Country where product is manufactured</v>
-      </c>
-      <c r="C7" t="str">
-        <v>India, China, USA</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MRP Quantity</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MRP printed quantity (e.g., 1L, 500g)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>500ML</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
-        <v>MRP Quantity</v>
-      </c>
-      <c r="B8" t="str">
-        <v>MRP printed quantity (e.g., 1L, 500g)</v>
-      </c>
-      <c r="C8" t="str">
-        <v>500ML</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Unit Type</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Unit of measurement</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UNIT, KG, LTR, ML, PCS</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
-        <v>Unit Type</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Unit of measurement</v>
-      </c>
-      <c r="C9" t="str">
-        <v>UNIT, KG, LTR, ML, PCS</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MRP</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Maximum Retail Price in INR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4999.00</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
-        <v>MRP</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Maximum Retail Price in INR</v>
-      </c>
-      <c r="C10" t="str">
-        <v>4999.00</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>USSP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Unit Standard Selling Price in INR</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3999.00</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
-        <v>USSP</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Unit Standard Selling Price in INR</v>
-      </c>
-      <c r="C11" t="str">
-        <v>3999.00</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Best Before (Months)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Shelf life in months</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
-        <v>Best Before (Months)</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Shelf life in months</v>
-      </c>
-      <c r="C12" t="str">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Factor</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Conversion factor for inventory</v>
-      </c>
-      <c r="C13" t="str">
-        <v>1</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Conversion factor for inventory</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>